<commit_message>
Preços das peças com link: aba Fontes e Orcamento_Pecas_Fontes.xlsx
Cada peça da Arquitetura A e do RFID futuro tem loja, produto, link e
preço consultados em 27/10/2026 (fontes_precos.py). Orçamentos completo,
POC e projeto interno, documento e apresentação regenerados com os
preços novos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TBWA3G7ku1j3oTf4VMkLud
</commit_message>
<xml_diff>
--- a/projeto/entregaveis/Orcamento_POC_PTL.xlsx
+++ b/projeto/entregaveis/Orcamento_POC_PTL.xlsx
@@ -1086,7 +1086,7 @@
       </c>
       <c r="B5" s="5" t="n">
         <f aca="false">'Fase 1 - Bancada'!E19</f>
-        <v>3347.65801774754</v>
+        <v>3447.13173520655</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>6</v>
@@ -1098,7 +1098,7 @@
       </c>
       <c r="B6" s="5" t="n">
         <f aca="false">'Fase 2 - Estações'!E40</f>
-        <v>17079.1306767491</v>
+        <v>17823.1651930606</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>8</v>
@@ -1110,7 +1110,7 @@
       </c>
       <c r="B7" s="8" t="n">
         <f aca="false">B5+B6</f>
-        <v>20426.7886944966</v>
+        <v>21270.2969282671</v>
       </c>
       <c r="C7" s="6"/>
     </row>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="B8" s="5" t="n">
         <f aca="false">B7*Premissas!$B$9</f>
-        <v>2042.67886944966</v>
+        <v>2127.02969282671</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>11</v>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="B9" s="10" t="n">
         <f aca="false">B7+B8</f>
-        <v>22469.4675639463</v>
+        <v>23397.3266210938</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>13</v>
@@ -1517,11 +1517,11 @@
         <v>1</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>549.810425</v>
+        <v>673.739525</v>
       </c>
       <c r="E5" s="22" t="n">
         <f aca="false">C5*D5</f>
-        <v>549.810425</v>
+        <v>673.739525</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1535,11 +1535,11 @@
         <v>1</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>96.8</v>
+        <v>117.59</v>
       </c>
       <c r="E6" s="22" t="n">
         <f aca="false">C6*D6</f>
-        <v>96.8</v>
+        <v>117.59</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1553,11 +1553,11 @@
         <v>4</v>
       </c>
       <c r="D7" s="16" t="n">
-        <v>45.1417049180328</v>
+        <v>55.2250459016394</v>
       </c>
       <c r="E7" s="22" t="n">
         <f aca="false">C7*D7</f>
-        <v>180.566819672131</v>
+        <v>220.900183606558</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1571,11 +1571,11 @@
         <v>2</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>134.95</v>
+        <v>151.48</v>
       </c>
       <c r="E8" s="22" t="n">
         <f aca="false">C8*D8</f>
-        <v>269.9</v>
+        <v>302.96</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1589,11 +1589,11 @@
         <v>1</v>
       </c>
       <c r="D9" s="16" t="n">
-        <v>45</v>
+        <v>25.611</v>
       </c>
       <c r="E9" s="22" t="n">
         <f aca="false">C9*D9</f>
-        <v>45</v>
+        <v>25.611</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1607,11 +1607,11 @@
         <v>20</v>
       </c>
       <c r="D10" s="16" t="n">
-        <v>4.03085245901639</v>
+        <v>2.62262295081967</v>
       </c>
       <c r="E10" s="22" t="n">
         <f aca="false">C10*D10</f>
-        <v>80.6170491803278</v>
+        <v>52.4524590163934</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1623,11 +1623,11 @@
         <v>20</v>
       </c>
       <c r="D11" s="16" t="n">
-        <v>0.8</v>
+        <v>0.7099</v>
       </c>
       <c r="E11" s="22" t="n">
         <f aca="false">C11*D11</f>
-        <v>16</v>
+        <v>14.198</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1641,11 +1641,11 @@
         <v>1</v>
       </c>
       <c r="D12" s="16" t="n">
-        <v>150</v>
+        <v>66.66</v>
       </c>
       <c r="E12" s="22" t="n">
         <f aca="false">C12*D12</f>
-        <v>150</v>
+        <v>66.66</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1659,11 +1659,11 @@
         <v>1</v>
       </c>
       <c r="D13" s="16" t="n">
-        <v>90</v>
+        <v>93.63</v>
       </c>
       <c r="E13" s="22" t="n">
         <f aca="false">C13*D13</f>
-        <v>90</v>
+        <v>93.63</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1695,11 +1695,11 @@
         <v>1</v>
       </c>
       <c r="D15" s="16" t="n">
-        <v>700</v>
+        <v>705.69</v>
       </c>
       <c r="E15" s="22" t="n">
         <f aca="false">C15*D15</f>
-        <v>700</v>
+        <v>705.69</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1716,7 +1716,7 @@
       </c>
       <c r="E16" s="22" t="n">
         <f aca="false">SUM(E5:E15)*D16</f>
-        <v>123.234214692623</v>
+        <v>127.971058381148</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1766,7 +1766,7 @@
       <c r="D19" s="25"/>
       <c r="E19" s="10" t="n">
         <f aca="false">SUM(E5:E18)</f>
-        <v>3347.65801774754</v>
+        <v>3447.13173520655</v>
       </c>
     </row>
   </sheetData>
@@ -1848,11 +1848,11 @@
         <v>71</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>45.1417049180328</v>
+        <v>55.2250459016394</v>
       </c>
       <c r="E6" s="22" t="n">
         <f aca="false">C6*D6</f>
-        <v>3205.06104918033</v>
+        <v>3920.9782590164</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1866,11 +1866,11 @@
         <v>22</v>
       </c>
       <c r="D7" s="16" t="n">
-        <v>96.8</v>
+        <v>117.59</v>
       </c>
       <c r="E7" s="22" t="n">
         <f aca="false">C7*D7</f>
-        <v>2129.6</v>
+        <v>2586.98</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1884,11 +1884,11 @@
         <v>14</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>134.95</v>
+        <v>151.48</v>
       </c>
       <c r="E8" s="22" t="n">
         <f aca="false">C8*D8</f>
-        <v>1889.3</v>
+        <v>2120.72</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1902,11 +1902,11 @@
         <v>3</v>
       </c>
       <c r="D9" s="16" t="n">
-        <v>549.810425</v>
+        <v>673.739525</v>
       </c>
       <c r="E9" s="22" t="n">
         <f aca="false">C9*D9</f>
-        <v>1649.431275</v>
+        <v>2021.218575</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1920,11 +1920,11 @@
         <v>120</v>
       </c>
       <c r="D10" s="16" t="n">
-        <v>4.03085245901639</v>
+        <v>2.62262295081967</v>
       </c>
       <c r="E10" s="22" t="n">
         <f aca="false">C10*D10</f>
-        <v>483.702295081967</v>
+        <v>314.71475409836</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1938,11 +1938,11 @@
         <v>72</v>
       </c>
       <c r="D11" s="16" t="n">
-        <v>0.8</v>
+        <v>0.7099</v>
       </c>
       <c r="E11" s="22" t="n">
         <f aca="false">C11*D11</f>
-        <v>57.6</v>
+        <v>51.1128</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1956,11 +1956,11 @@
         <v>54</v>
       </c>
       <c r="D12" s="16" t="n">
-        <v>9</v>
+        <v>4.36</v>
       </c>
       <c r="E12" s="22" t="n">
         <f aca="false">C12*D12</f>
-        <v>486</v>
+        <v>235.44</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1974,11 +1974,11 @@
         <v>2</v>
       </c>
       <c r="D13" s="16" t="n">
-        <v>40</v>
+        <v>28.52</v>
       </c>
       <c r="E13" s="22" t="n">
         <f aca="false">C13*D13</f>
-        <v>80</v>
+        <v>57.04</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1992,11 +1992,11 @@
         <v>2</v>
       </c>
       <c r="D14" s="16" t="n">
-        <v>45</v>
+        <v>25.611</v>
       </c>
       <c r="E14" s="22" t="n">
         <f aca="false">C14*D14</f>
-        <v>90</v>
+        <v>51.222</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2010,11 +2010,11 @@
         <v>100</v>
       </c>
       <c r="D15" s="16" t="n">
-        <v>4.03085245901639</v>
+        <v>2.62262295081967</v>
       </c>
       <c r="E15" s="22" t="n">
         <f aca="false">C15*D15</f>
-        <v>403.085245901639</v>
+        <v>262.262295081967</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2064,11 +2064,11 @@
         <v>1</v>
       </c>
       <c r="D18" s="16" t="n">
-        <v>550</v>
+        <v>431.08</v>
       </c>
       <c r="E18" s="22" t="n">
         <f aca="false">C18*D18</f>
-        <v>550</v>
+        <v>431.08</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2082,11 +2082,11 @@
         <v>80</v>
       </c>
       <c r="D19" s="16" t="n">
-        <v>4.03085245901639</v>
+        <v>2.62262295081967</v>
       </c>
       <c r="E19" s="22" t="n">
         <f aca="false">C19*D19</f>
-        <v>322.468196721311</v>
+        <v>209.809836065574</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2136,11 +2136,11 @@
         <v>1</v>
       </c>
       <c r="D22" s="16" t="n">
-        <v>700</v>
+        <v>705.69</v>
       </c>
       <c r="E22" s="22" t="n">
         <f aca="false">C22*D22</f>
-        <v>700</v>
+        <v>705.69</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2157,7 +2157,7 @@
       </c>
       <c r="E23" s="22" t="n">
         <f aca="false">SUM(E6:E22)*D23</f>
-        <v>690.982903094262</v>
+        <v>737.083925963115</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2169,7 +2169,7 @@
       <c r="D24" s="25"/>
       <c r="E24" s="10" t="n">
         <f aca="false">SUM(E6:E23)</f>
-        <v>14510.6409649795</v>
+        <v>15478.7624452254</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2365,7 +2365,7 @@
       <c r="D38" s="4"/>
       <c r="E38" s="5" t="n">
         <f aca="false">-('Fase 1 - Bancada'!E14+'Fase 1 - Bancada'!E15)*(1+Premissas!$B$8)</f>
-        <v>-1035.2895</v>
+        <v>-1041.264</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2379,7 +2379,7 @@
       <c r="D39" s="4"/>
       <c r="E39" s="5" t="n">
         <f aca="false">-('Fase 1 - Bancada'!E5+'Fase 1 - Bancada'!E6+'Fase 1 - Bancada'!E7+'Fase 1 - Bancada'!E8)</f>
-        <v>-1097.07724467213</v>
+        <v>-1315.18970860656</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2391,7 +2391,7 @@
       <c r="D40" s="25"/>
       <c r="E40" s="10" t="n">
         <f aca="false">E24+E35+E38+E39</f>
-        <v>17079.1306767491</v>
+        <v>17823.1651930606</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Carcaças dos LEDs em 3D com valor estipulado; RFID em abas separadas
P13 e P14 voltam a valor estipulado (impressão 3D, medida padrão compacta).
Fontes e peças do RFID futuro ficam em abas próprias, sem misturar com o
projeto. Orçamentos, documento e apresentação regenerados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TBWA3G7ku1j3oTf4VMkLud
</commit_message>
<xml_diff>
--- a/projeto/entregaveis/Orcamento_POC_PTL.xlsx
+++ b/projeto/entregaveis/Orcamento_POC_PTL.xlsx
@@ -1086,7 +1086,7 @@
       </c>
       <c r="B5" s="5" t="n">
         <f aca="false">'Fase 1 - Bancada'!E19</f>
-        <v>3447.13173520655</v>
+        <v>3374.81823520655</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>6</v>
@@ -1098,7 +1098,7 @@
       </c>
       <c r="B6" s="5" t="n">
         <f aca="false">'Fase 2 - Estações'!E40</f>
-        <v>17823.1651930606</v>
+        <v>16847.0121930606</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>8</v>
@@ -1110,7 +1110,7 @@
       </c>
       <c r="B7" s="8" t="n">
         <f aca="false">B5+B6</f>
-        <v>21270.2969282671</v>
+        <v>20221.8304282671</v>
       </c>
       <c r="C7" s="6"/>
     </row>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="B8" s="5" t="n">
         <f aca="false">B7*Premissas!$B$9</f>
-        <v>2127.02969282671</v>
+        <v>2022.18304282671</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>11</v>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="B9" s="10" t="n">
         <f aca="false">B7+B8</f>
-        <v>23397.3266210938</v>
+        <v>22244.0134710938</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>13</v>
@@ -1535,11 +1535,11 @@
         <v>1</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>117.59</v>
+        <v>104.42</v>
       </c>
       <c r="E6" s="22" t="n">
         <f aca="false">C6*D6</f>
-        <v>117.59</v>
+        <v>104.42</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1553,11 +1553,11 @@
         <v>4</v>
       </c>
       <c r="D7" s="16" t="n">
-        <v>55.2250459016394</v>
+        <v>47.8850459016393</v>
       </c>
       <c r="E7" s="22" t="n">
         <f aca="false">C7*D7</f>
-        <v>220.900183606558</v>
+        <v>191.540183606557</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1571,11 +1571,11 @@
         <v>2</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>151.48</v>
+        <v>138.31</v>
       </c>
       <c r="E8" s="22" t="n">
         <f aca="false">C8*D8</f>
-        <v>302.96</v>
+        <v>276.62</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1716,7 +1716,7 @@
       </c>
       <c r="E16" s="22" t="n">
         <f aca="false">SUM(E5:E15)*D16</f>
-        <v>127.971058381148</v>
+        <v>124.527558381148</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1766,7 +1766,7 @@
       <c r="D19" s="25"/>
       <c r="E19" s="10" t="n">
         <f aca="false">SUM(E5:E18)</f>
-        <v>3447.13173520655</v>
+        <v>3374.81823520655</v>
       </c>
     </row>
   </sheetData>
@@ -1848,11 +1848,11 @@
         <v>71</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>55.2250459016394</v>
+        <v>47.8850459016393</v>
       </c>
       <c r="E6" s="22" t="n">
         <f aca="false">C6*D6</f>
-        <v>3920.9782590164</v>
+        <v>3399.83825901639</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1866,11 +1866,11 @@
         <v>22</v>
       </c>
       <c r="D7" s="16" t="n">
-        <v>117.59</v>
+        <v>104.42</v>
       </c>
       <c r="E7" s="22" t="n">
         <f aca="false">C7*D7</f>
-        <v>2586.98</v>
+        <v>2297.24</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1884,11 +1884,11 @@
         <v>14</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>151.48</v>
+        <v>138.31</v>
       </c>
       <c r="E8" s="22" t="n">
         <f aca="false">C8*D8</f>
-        <v>2120.72</v>
+        <v>1936.34</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2157,7 +2157,7 @@
       </c>
       <c r="E23" s="22" t="n">
         <f aca="false">SUM(E6:E22)*D23</f>
-        <v>737.083925963115</v>
+        <v>687.320925963115</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2169,7 +2169,7 @@
       <c r="D24" s="25"/>
       <c r="E24" s="10" t="n">
         <f aca="false">SUM(E6:E23)</f>
-        <v>15478.7624452254</v>
+        <v>14433.7394452254</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2379,7 +2379,7 @@
       <c r="D39" s="4"/>
       <c r="E39" s="5" t="n">
         <f aca="false">-('Fase 1 - Bancada'!E5+'Fase 1 - Bancada'!E6+'Fase 1 - Bancada'!E7+'Fase 1 - Bancada'!E8)</f>
-        <v>-1315.18970860656</v>
+        <v>-1246.31970860656</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2391,7 +2391,7 @@
       <c r="D40" s="25"/>
       <c r="E40" s="10" t="n">
         <f aca="false">E24+E35+E38+E39</f>
-        <v>17823.1651930606</v>
+        <v>16847.0121930606</v>
       </c>
     </row>
   </sheetData>

</xml_diff>